<commit_message>
Updated EPA VOC mapping for our mechanisms
</commit_message>
<xml_diff>
--- a/Hawthorne_data/epa_parameters_reference.xlsx
+++ b/Hawthorne_data/epa_parameters_reference.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/Hawthorne_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EE8EF3-A4A7-F043-AB0C-702DC6111D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B18F06B7-93A7-DF46-9ECF-3FA3E79DB128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="980" yWindow="740" windowWidth="25960" windowHeight="20140" xr2:uid="{34C1F88B-7F25-2A44-9437-4479E7A58C96}"/>
+    <workbookView xWindow="37640" yWindow="540" windowWidth="32700" windowHeight="21040" xr2:uid="{34C1F88B-7F25-2A44-9437-4479E7A58C96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -626,10 +626,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -949,1242 +948,1240 @@
   <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="2"/>
-    <col min="2" max="2" width="24.33203125" style="2" customWidth="1"/>
-    <col min="3" max="4" width="10.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.1640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="20" style="2" customWidth="1"/>
-    <col min="8" max="8" width="28" style="2" customWidth="1"/>
-    <col min="9" max="9" width="31" style="2" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="24.33203125" customWidth="1"/>
+    <col min="3" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.1640625" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="31" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>142</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>118</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>121</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>143</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>154</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>161</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="A2">
         <v>43102</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+      <c r="A3">
         <v>43141</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4">
         <v>43202</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>122</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" t="s">
         <v>139</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" t="s">
         <v>145</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="2" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="A5">
         <v>43203</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>165</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" t="s">
         <v>145</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
+      <c r="A6">
         <v>43204</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
         <v>78</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" t="s">
         <v>141</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="K6" s="3" t="s">
+      <c r="G6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>43205</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>167</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" t="s">
         <v>166</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="A8">
         <v>43206</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>146</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" t="s">
         <v>145</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
+      <c r="A9">
         <v>43212</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10">
         <v>43214</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
         <v>90</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+      <c r="A11">
         <v>43216</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
         <v>37</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H11" s="2" t="s">
+      <c r="G11" t="s">
+        <v>144</v>
+      </c>
+      <c r="H11" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="A12">
         <v>43217</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
         <v>31</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H12" s="2" t="s">
+      <c r="G12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H12" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13">
         <v>43218</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
         <v>114</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" t="s">
         <v>147</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
+      <c r="A14">
         <v>43220</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>125</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
+      <c r="A15">
         <v>43221</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
         <v>57</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="A16">
         <v>43224</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
         <v>49</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H16" s="2" t="s">
+      <c r="G16" t="s">
+        <v>144</v>
+      </c>
+      <c r="H16" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+      <c r="A17">
         <v>43226</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
         <v>94</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H17" s="2" t="s">
+      <c r="G17" t="s">
+        <v>144</v>
+      </c>
+      <c r="H17" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="2">
+      <c r="A18">
         <v>43227</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
         <v>111</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H18" s="2" t="s">
+      <c r="G18" t="s">
+        <v>144</v>
+      </c>
+      <c r="H18" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
+      <c r="A19">
         <v>43230</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
         <v>101</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
+      <c r="A20">
         <v>43231</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" t="s">
         <v>126</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="2">
+      <c r="A21">
         <v>43232</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" t="s">
         <v>100</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
+      <c r="A22">
         <v>43233</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
+      <c r="A23">
         <v>43235</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
+      <c r="A24">
         <v>43238</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" t="s">
         <v>85</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" t="s">
         <v>149</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A25" s="2">
+      <c r="A25">
         <v>43242</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" t="s">
         <v>115</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="2">
+      <c r="A26">
         <v>43243</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" t="s">
         <v>130</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" t="s">
         <v>150</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" t="s">
         <v>145</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
+      <c r="A27">
         <v>43244</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
+      <c r="A28">
         <v>43245</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28" t="s">
         <v>39</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H28" s="2" t="s">
+      <c r="G28" t="s">
+        <v>144</v>
+      </c>
+      <c r="H28" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29" s="2">
+      <c r="A29">
         <v>43247</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="C29" t="s">
+        <v>3</v>
+      </c>
+      <c r="D29" t="s">
         <v>102</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="G29" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" s="2">
+      <c r="A30">
         <v>43248</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="C30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D30" t="s">
         <v>93</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="2">
+      <c r="A31">
         <v>43249</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="C31" t="s">
+        <v>3</v>
+      </c>
+      <c r="D31" t="s">
         <v>106</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G31" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="2">
+      <c r="A32">
         <v>43250</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="C32" t="s">
+        <v>3</v>
+      </c>
+      <c r="D32" t="s">
         <v>112</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" s="2">
+      <c r="A33">
         <v>43252</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="C33" t="s">
+        <v>3</v>
+      </c>
+      <c r="D33" t="s">
         <v>96</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="2">
+      <c r="A34">
         <v>43253</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="C34" t="s">
+        <v>3</v>
+      </c>
+      <c r="D34" t="s">
         <v>41</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
+      <c r="A35">
         <v>43261</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="C35" t="s">
+        <v>3</v>
+      </c>
+      <c r="D35" t="s">
         <v>116</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
+      <c r="A36">
         <v>43262</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" t="s">
         <v>22</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="C36" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" t="s">
         <v>109</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
+      <c r="A37">
         <v>43263</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" t="s">
         <v>76</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="C37" t="s">
+        <v>3</v>
+      </c>
+      <c r="D37" t="s">
         <v>77</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="G37" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
+      <c r="A38">
         <v>43280</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" t="s">
         <v>23</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="C38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
         <v>110</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H38" s="2" t="s">
+      <c r="G38" t="s">
+        <v>144</v>
+      </c>
+      <c r="H38" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
+      <c r="A39">
         <v>43284</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" t="s">
         <v>66</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D39" s="2" t="s">
+      <c r="C39" t="s">
+        <v>3</v>
+      </c>
+      <c r="D39" t="s">
         <v>67</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G39" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
+      <c r="A40">
         <v>43285</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D40" s="2" t="s">
+      <c r="C40" t="s">
+        <v>3</v>
+      </c>
+      <c r="D40" t="s">
         <v>55</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="G40" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
+      <c r="A41">
         <v>43291</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D41" s="2" t="s">
+      <c r="C41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" t="s">
         <v>59</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G41" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
+      <c r="A42">
         <v>43502</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="C42" t="s">
+        <v>3</v>
+      </c>
+      <c r="D42" t="s">
         <v>89</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" t="s">
         <v>137</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="F42" t="s">
         <v>152</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="G42" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A43" s="2">
+      <c r="A43">
         <v>43954</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D43" s="2" t="s">
+      <c r="C43" t="s">
+        <v>3</v>
+      </c>
+      <c r="D43" t="s">
         <v>97</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="G43" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" s="2">
+      <c r="A44">
         <v>43960</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" t="s">
         <v>18</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D44" s="2" t="s">
+      <c r="C44" t="s">
+        <v>3</v>
+      </c>
+      <c r="D44" t="s">
         <v>105</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="G44" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" s="2">
+      <c r="A45">
         <v>45109</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" t="s">
         <v>70</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D45" s="2" t="s">
+      <c r="C45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D45" t="s">
         <v>71</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" t="s">
         <v>133</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" t="s">
         <v>153</v>
       </c>
-      <c r="G45" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H45" s="2" t="s">
+      <c r="G45" t="s">
+        <v>144</v>
+      </c>
+      <c r="H45" t="s">
         <v>155</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="K45" t="s">
         <v>153</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="L45" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A46" s="2">
+      <c r="A46">
         <v>45201</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" t="s">
         <v>4</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D46" s="2" t="s">
+      <c r="C46" t="s">
+        <v>3</v>
+      </c>
+      <c r="D46" t="s">
         <v>91</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="E46" t="s">
         <v>131</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F46" t="s">
         <v>156</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="G46" t="s">
         <v>145</v>
       </c>
-      <c r="K46" s="2" t="s">
+      <c r="K46" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A47" s="2">
+      <c r="A47">
         <v>45202</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" t="s">
         <v>26</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D47" s="2" t="s">
+      <c r="C47" t="s">
+        <v>3</v>
+      </c>
+      <c r="D47" t="s">
         <v>113</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="E47" t="s">
         <v>132</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" t="s">
         <v>158</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="G47" t="s">
         <v>145</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="K47" t="s">
         <v>158</v>
       </c>
-      <c r="L47" s="2" t="s">
+      <c r="L47" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
+      <c r="A48">
         <v>45203</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" t="s">
         <v>46</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D48" s="2" t="s">
+      <c r="C48" t="s">
+        <v>3</v>
+      </c>
+      <c r="D48" t="s">
         <v>47</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" t="s">
         <v>120</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" t="s">
         <v>157</v>
       </c>
-      <c r="G48" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="K48" s="2" t="s">
+      <c r="G48" t="s">
+        <v>144</v>
+      </c>
+      <c r="K48" t="s">
         <v>153</v>
       </c>
-      <c r="L48" s="2" t="s">
+      <c r="L48" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" s="2">
+      <c r="A49">
         <v>45204</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D49" s="2" t="s">
+      <c r="C49" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" t="s">
         <v>51</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" t="s">
         <v>136</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" t="s">
         <v>153</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H49" s="2" t="s">
+      <c r="G49" t="s">
+        <v>144</v>
+      </c>
+      <c r="H49" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A50" s="2">
+      <c r="A50">
         <v>45207</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D50" s="2" t="s">
+      <c r="C50" t="s">
+        <v>3</v>
+      </c>
+      <c r="D50" t="s">
         <v>87</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="2">
+      <c r="A51">
         <v>45208</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" t="s">
         <v>17</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D51" s="2" t="s">
+      <c r="C51" t="s">
+        <v>3</v>
+      </c>
+      <c r="D51" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" s="2">
+      <c r="A52">
         <v>45209</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D52" s="2" t="s">
+      <c r="C52" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="2">
+      <c r="A53">
         <v>45210</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" t="s">
         <v>5</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D53" s="2" t="s">
+      <c r="C53" t="s">
+        <v>3</v>
+      </c>
+      <c r="D53" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" s="2">
+      <c r="A54">
         <v>45211</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" t="s">
         <v>12</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D54" s="2" t="s">
+      <c r="C54" t="s">
+        <v>3</v>
+      </c>
+      <c r="D54" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A55" s="2">
+      <c r="A55">
         <v>45212</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" t="s">
         <v>19</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D55" s="2" t="s">
+      <c r="C55" t="s">
+        <v>3</v>
+      </c>
+      <c r="D55" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A56" s="2">
+      <c r="A56">
         <v>45213</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" t="s">
         <v>32</v>
       </c>
-      <c r="C56" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D56" s="2" t="s">
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" s="2">
+      <c r="A57">
         <v>45218</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D57" s="2" t="s">
+      <c r="C57" t="s">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A58" s="2">
+      <c r="A58">
         <v>45219</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" t="s">
         <v>16</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D58" s="2" t="s">
+      <c r="C58" t="s">
+        <v>3</v>
+      </c>
+      <c r="D58" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A59" s="2">
+      <c r="A59">
         <v>45220</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" t="s">
         <v>52</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D59" s="2" t="s">
+      <c r="C59" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" t="s">
         <v>53</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" t="s">
         <v>160</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" t="s">
         <v>159</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="G59" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" s="2">
+      <c r="A60">
         <v>45225</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D60" s="2" t="s">
+      <c r="C60" t="s">
+        <v>3</v>
+      </c>
+      <c r="D60" t="s">
         <v>73</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed random tab spaces from CAS numbers of Hawthorne EPA VOC data when copy pasted
</commit_message>
<xml_diff>
--- a/Hawthorne_data/epa_parameters_reference.xlsx
+++ b/Hawthorne_data/epa_parameters_reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/Hawthorne_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Documents\GitHub\USOS_shared\Hawthorne_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B18F06B7-93A7-DF46-9ECF-3FA3E79DB128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96FE3B8-BA85-4BB3-84F1-227CEBD6EC66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37640" yWindow="540" windowWidth="32700" windowHeight="21040" xr2:uid="{34C1F88B-7F25-2A44-9437-4479E7A58C96}"/>
+    <workbookView xWindow="10176" yWindow="2652" windowWidth="12684" windowHeight="8880" xr2:uid="{34C1F88B-7F25-2A44-9437-4479E7A58C96}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -27,9 +27,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -167,9 +168,6 @@
     <t>n-Pentane</t>
   </si>
   <si>
-    <t xml:space="preserve">	109-66-0</t>
-  </si>
-  <si>
     <t>n-Propylbenzene</t>
   </si>
   <si>
@@ -233,9 +231,6 @@
     <t>Ethylene</t>
   </si>
   <si>
-    <t xml:space="preserve">	74-85-1</t>
-  </si>
-  <si>
     <t>2,3-Dimethylbutane</t>
   </si>
   <si>
@@ -311,15 +306,6 @@
     <t>75-28-5</t>
   </si>
   <si>
-    <t xml:space="preserve">	71-43-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">98-82-8	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	110-82-7</t>
-  </si>
-  <si>
     <t>646-04-8</t>
   </si>
   <si>
@@ -329,21 +315,12 @@
     <t>565-75-3</t>
   </si>
   <si>
-    <t xml:space="preserve">	1120-21-4</t>
-  </si>
-  <si>
     <t>115-07-1</t>
   </si>
   <si>
-    <t xml:space="preserve">	611-14-3</t>
-  </si>
-  <si>
     <t xml:space="preserve">142-82-5	</t>
   </si>
   <si>
-    <t xml:space="preserve">	96-14-0</t>
-  </si>
-  <si>
     <t>108-08-7</t>
   </si>
   <si>
@@ -362,9 +339,6 @@
     <t xml:space="preserve">620-14-4	</t>
   </si>
   <si>
-    <t xml:space="preserve">	112-40-3</t>
-  </si>
-  <si>
     <t xml:space="preserve">96-37-7	</t>
   </si>
   <si>
@@ -374,9 +348,6 @@
     <t xml:space="preserve">	627-20-3</t>
   </si>
   <si>
-    <t xml:space="preserve">	540-84-1</t>
-  </si>
-  <si>
     <t>108-88-3</t>
   </si>
   <si>
@@ -573,6 +544,36 @@
   </si>
   <si>
     <t>BENZ</t>
+  </si>
+  <si>
+    <t>112-40-3</t>
+  </si>
+  <si>
+    <t>611-14-3</t>
+  </si>
+  <si>
+    <t>98-82-8</t>
+  </si>
+  <si>
+    <t>71-43-2</t>
+  </si>
+  <si>
+    <t>1120-21-4</t>
+  </si>
+  <si>
+    <t>74-85-1</t>
+  </si>
+  <si>
+    <t>109-66-0</t>
+  </si>
+  <si>
+    <t>540-84-1</t>
+  </si>
+  <si>
+    <t>96-14-0</t>
+  </si>
+  <si>
+    <t>110-82-7</t>
   </si>
 </sst>
 </file>
@@ -946,65 +947,65 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42CE89AC-9EDC-D444-96A1-49660B75F03A}">
   <dimension ref="A1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="24.33203125" customWidth="1"/>
-    <col min="3" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="21.1640625" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.296875" customWidth="1"/>
+    <col min="3" max="4" width="10.796875" customWidth="1"/>
+    <col min="5" max="5" width="21.19921875" customWidth="1"/>
+    <col min="6" max="6" width="19.796875" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
     <col min="9" max="9" width="31" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E1" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="F1" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="G1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="H1" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="I1" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="K1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>43102</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>43141</v>
       </c>
@@ -1015,10 +1016,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>43202</v>
       </c>
@@ -1029,74 +1030,74 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="F4" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G4" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>43203</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>174</v>
       </c>
       <c r="E5" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="F5" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>43204</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
         <v>3</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="G6" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>43205</v>
       </c>
@@ -1107,19 +1108,19 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="F7" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>43206</v>
       </c>
@@ -1133,36 +1134,36 @@
         <v>35</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="F8" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="G8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>43212</v>
       </c>
       <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
         <v>62</v>
       </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" t="s">
-        <v>63</v>
-      </c>
       <c r="E9" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>43214</v>
       </c>
@@ -1173,13 +1174,13 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>43216</v>
       </c>
@@ -1193,16 +1194,16 @@
         <v>37</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G11" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H11" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>43217</v>
       </c>
@@ -1216,16 +1217,16 @@
         <v>31</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G12" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H12" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>43218</v>
       </c>
@@ -1236,16 +1237,16 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="G13" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>43220</v>
       </c>
@@ -1256,62 +1257,62 @@
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>175</v>
       </c>
       <c r="E14" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="G14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>43221</v>
       </c>
       <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
         <v>56</v>
       </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>57</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>43224</v>
       </c>
       <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
         <v>48</v>
       </c>
-      <c r="C16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" t="s">
-        <v>49</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="G16" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H16" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>43226</v>
       </c>
@@ -1322,19 +1323,19 @@
         <v>3</v>
       </c>
       <c r="D17" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G17" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H17" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>43227</v>
       </c>
@@ -1345,19 +1346,19 @@
         <v>3</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G18" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H18" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>43230</v>
       </c>
@@ -1368,36 +1369,36 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
+        <v>177</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G19" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>43231</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
         <v>3</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="H20" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>43232</v>
       </c>
@@ -1408,67 +1409,67 @@
         <v>3</v>
       </c>
       <c r="D21" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>43233</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
         <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>43235</v>
       </c>
       <c r="B23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
         <v>60</v>
       </c>
-      <c r="C23" t="s">
-        <v>3</v>
-      </c>
-      <c r="D23" t="s">
-        <v>61</v>
-      </c>
       <c r="E23" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>43238</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
         <v>3</v>
       </c>
       <c r="D24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F24" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="G24" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>43242</v>
       </c>
@@ -1479,42 +1480,42 @@
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="G25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>43243</v>
       </c>
       <c r="B26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
         <v>3</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E26" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G26" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K26" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>43244</v>
       </c>
@@ -1525,10 +1526,10 @@
         <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>43245</v>
       </c>
@@ -1542,16 +1543,16 @@
         <v>39</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="G28" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H28" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>43247</v>
       </c>
@@ -1562,16 +1563,16 @@
         <v>3</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G29" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>43248</v>
       </c>
@@ -1582,16 +1583,16 @@
         <v>3</v>
       </c>
       <c r="D30" t="s">
-        <v>93</v>
+        <v>178</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G30" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>43249</v>
       </c>
@@ -1602,16 +1603,16 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G31" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>43250</v>
       </c>
@@ -1622,16 +1623,16 @@
         <v>3</v>
       </c>
       <c r="D32" t="s">
-        <v>112</v>
+        <v>176</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G32" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>43252</v>
       </c>
@@ -1642,16 +1643,16 @@
         <v>3</v>
       </c>
       <c r="D33" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G33" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>43253</v>
       </c>
@@ -1665,33 +1666,33 @@
         <v>41</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G34" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>43261</v>
       </c>
       <c r="B35" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C35" t="s">
         <v>3</v>
       </c>
       <c r="D35" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G35" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>43262</v>
       </c>
@@ -1702,36 +1703,36 @@
         <v>3</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G36" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>43263</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C37" t="s">
         <v>3</v>
       </c>
       <c r="D37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G37" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>43280</v>
       </c>
@@ -1742,102 +1743,102 @@
         <v>3</v>
       </c>
       <c r="D38" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="G38" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H38" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>43284</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C39" t="s">
         <v>3</v>
       </c>
       <c r="D39" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G39" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>43285</v>
       </c>
       <c r="B40" t="s">
+        <v>53</v>
+      </c>
+      <c r="C40" t="s">
+        <v>3</v>
+      </c>
+      <c r="D40" t="s">
         <v>54</v>
       </c>
-      <c r="C40" t="s">
-        <v>3</v>
-      </c>
-      <c r="D40" t="s">
-        <v>55</v>
-      </c>
       <c r="F40" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G40" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>43291</v>
       </c>
       <c r="B41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" t="s">
         <v>58</v>
       </c>
-      <c r="C41" t="s">
-        <v>3</v>
-      </c>
-      <c r="D41" t="s">
-        <v>59</v>
-      </c>
       <c r="F41" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G41" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>43502</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C42" t="s">
         <v>3</v>
       </c>
       <c r="D42" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E42" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="F42" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="G42" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>43954</v>
       </c>
@@ -1848,16 +1849,16 @@
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>97</v>
+        <v>173</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G43" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43960</v>
       </c>
@@ -1868,48 +1869,48 @@
         <v>3</v>
       </c>
       <c r="D44" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G44" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>45109</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C45" t="s">
         <v>3</v>
       </c>
       <c r="D45" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E45" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="F45" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="G45" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H45" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="K45" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="L45" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45201</v>
       </c>
@@ -1920,22 +1921,22 @@
         <v>3</v>
       </c>
       <c r="D46" t="s">
-        <v>91</v>
+        <v>172</v>
       </c>
       <c r="E46" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="F46" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="G46" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K46" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45202</v>
       </c>
@@ -1946,97 +1947,97 @@
         <v>3</v>
       </c>
       <c r="D47" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="E47" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="F47" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="G47" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="K47" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="L47" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>45203</v>
       </c>
       <c r="B48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C48" t="s">
+        <v>3</v>
+      </c>
+      <c r="D48" t="s">
         <v>46</v>
       </c>
-      <c r="C48" t="s">
-        <v>3</v>
-      </c>
-      <c r="D48" t="s">
-        <v>47</v>
-      </c>
       <c r="E48" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="F48" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="G48" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="K48" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="L48" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>45204</v>
       </c>
       <c r="B49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" t="s">
         <v>50</v>
       </c>
-      <c r="C49" t="s">
-        <v>3</v>
-      </c>
-      <c r="D49" t="s">
-        <v>51</v>
-      </c>
       <c r="E49" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="F49" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="G49" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H49" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>45207</v>
       </c>
       <c r="B50" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C50" t="s">
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E50" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>45208</v>
       </c>
@@ -2047,24 +2048,24 @@
         <v>3</v>
       </c>
       <c r="D51" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>45209</v>
       </c>
       <c r="B52" t="s">
+        <v>43</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
         <v>44</v>
       </c>
-      <c r="C52" t="s">
-        <v>3</v>
-      </c>
-      <c r="D52" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>45210</v>
       </c>
@@ -2075,10 +2076,10 @@
         <v>3</v>
       </c>
       <c r="D53" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>45211</v>
       </c>
@@ -2089,10 +2090,10 @@
         <v>3</v>
       </c>
       <c r="D54" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>45212</v>
       </c>
@@ -2103,10 +2104,10 @@
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>45213</v>
       </c>
@@ -2120,21 +2121,21 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>45218</v>
       </c>
       <c r="B57" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C57" t="s">
         <v>3</v>
       </c>
       <c r="D57" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>45219</v>
       </c>
@@ -2145,44 +2146,44 @@
         <v>3</v>
       </c>
       <c r="D58" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>45220</v>
       </c>
       <c r="B59" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" t="s">
         <v>52</v>
       </c>
-      <c r="C59" t="s">
-        <v>3</v>
-      </c>
-      <c r="D59" t="s">
-        <v>53</v>
-      </c>
       <c r="E59" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F59" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G59" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>45225</v>
       </c>
       <c r="B60" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C60" t="s">
         <v>3</v>
       </c>
       <c r="D60" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>